<commit_message>
cleaning up old code and updating data files
</commit_message>
<xml_diff>
--- a/docs/Mech Data.xlsx
+++ b/docs/Mech Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FoundryData-Dev\Data\systems\mwd\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961015C9-46B8-42CA-974E-71A6DF59CF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8326161-EC90-4AEF-B148-CBFC075BCF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22440" yWindow="2175" windowWidth="24885" windowHeight="19275" xr2:uid="{8D44F242-D0B2-4B9E-94CF-33F11494976A}"/>
+    <workbookView xWindow="51480" yWindow="-4995" windowWidth="16440" windowHeight="28320" xr2:uid="{8D44F242-D0B2-4B9E-94CF-33F11494976A}"/>
   </bookViews>
   <sheets>
     <sheet name="Mechs" sheetId="1" r:id="rId1"/>
@@ -1618,9 +1618,15 @@
       <c r="N4" s="12">
         <v>4</v>
       </c>
-      <c r="O4" s="12"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="12"/>
+      <c r="O4" s="12">
+        <v>3</v>
+      </c>
+      <c r="P4" s="1">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="12">
+        <v>3</v>
+      </c>
       <c r="R4" s="3">
         <v>1728000</v>
       </c>

</xml_diff>

<commit_message>
Implement melee attack resolution
</commit_message>
<xml_diff>
--- a/docs/Mech Data.xlsx
+++ b/docs/Mech Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FoundryData-Dev\Data\systems\mwd\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10FBC4AF-F6F2-43DD-860F-6EEE9C0A8CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E516EFF-50DE-4984-80EA-ABC96E607761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-4995" windowWidth="16440" windowHeight="28320" xr2:uid="{8D44F242-D0B2-4B9E-94CF-33F11494976A}"/>
+    <workbookView xWindow="27240" yWindow="1050" windowWidth="23205" windowHeight="19275" activeTab="2" xr2:uid="{8D44F242-D0B2-4B9E-94CF-33F11494976A}"/>
   </bookViews>
   <sheets>
     <sheet name="Mechs" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="497">
   <si>
     <t>Chassis</t>
   </si>
@@ -794,12 +794,6 @@
     <t>Reinforced Cockpit</t>
   </si>
   <si>
-    <t>Modules</t>
-  </si>
-  <si>
-    <t>Quirks</t>
-  </si>
-  <si>
     <t>Low Profile</t>
   </si>
   <si>
@@ -887,9 +881,6 @@
     <t>Combat  Electronics</t>
   </si>
   <si>
-    <t>Hardened Structure Components</t>
-  </si>
-  <si>
     <t>Advanced Optics</t>
   </si>
   <si>
@@ -899,6 +890,9 @@
     <t>Jump Booster</t>
   </si>
   <si>
+    <t>Thermal Exchanger</t>
+  </si>
+  <si>
     <t>Thermal Bank</t>
   </si>
   <si>
@@ -935,15 +929,9 @@
     <t>Electronic Protection Array</t>
   </si>
   <si>
-    <t>UAV Integration Compartment</t>
-  </si>
-  <si>
     <t>Hardened Armor</t>
   </si>
   <si>
-    <t>Laser Heat Sink</t>
-  </si>
-  <si>
     <t>Reactive Plating</t>
   </si>
   <si>
@@ -1147,9 +1135,6 @@
     <t>speedBoost, legs, heat</t>
   </si>
   <si>
-    <t>-1 trackingPenalty</t>
-  </si>
-  <si>
     <t>Generates +1 heat when used</t>
   </si>
   <si>
@@ -2800,9 +2785,6 @@
     <t>Targeting/Attack; Mobility Provider</t>
   </si>
   <si>
-    <t>Improved Actuators Mechanics</t>
-  </si>
-  <si>
     <t xml:space="preserve">Packrat </t>
   </si>
   <si>
@@ -2903,6 +2885,609 @@
   </si>
   <si>
     <t>Cruiser</t>
+  </si>
+  <si>
+    <t>Machine Quirks</t>
+  </si>
+  <si>
+    <t>Heat disappation unaffected by environmental factors</t>
+  </si>
+  <si>
+    <t>+1 heatProfile</t>
+  </si>
+  <si>
+    <t>+1 heatDissapation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armor gains 2 Concussive Resistance </t>
+  </si>
+  <si>
+    <t>Armor gains 2 Energy Resistance</t>
+  </si>
+  <si>
+    <t>Armor gains 2 Penatrating Resistance</t>
+  </si>
+  <si>
+    <t>Asset Modules</t>
+  </si>
+  <si>
+    <t>Anti-Missile System</t>
+  </si>
+  <si>
+    <t>Laser AMS</t>
+  </si>
+  <si>
+    <t>Laser Heat Sinks</t>
+  </si>
+  <si>
+    <t>Hardened Structural Components</t>
+  </si>
+  <si>
+    <t>UAV Control Pod</t>
+  </si>
+  <si>
+    <t>Missile Cluster Dice hit on 6</t>
+  </si>
+  <si>
+    <t>High Emission: Enemies reduce trackingPenalty against this machine by 1, minimum 0. Enemies gain +1 die to acquireTarget against this machine when emissions are relevant.</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>High Emission [Rating]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Enemies reduce trackingPenalty against this machine by [Rating], minimum 0. Enemies gain +[Rating] die to acquireTarget against this machine when emissions are relevant.</t>
+  </si>
+  <si>
+    <t>High Emission (1)</t>
+  </si>
+  <si>
+    <t>Volatile component or ammo explosion event</t>
+  </si>
+  <si>
+    <t>CASE destroyed/consumed when it prevents a catastrophic event.</t>
+  </si>
+  <si>
+    <t>Prevents full machine destruction and automatic crew death. Local location still suffers severe consequence: condition +1, stress spike, or module destruction.</t>
+  </si>
+  <si>
+    <r>
+      <t>+2 dice</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>feedReset</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and other Feed-related remedies. Applies to Jammed Ballistic, Ammo Feed Fault, Weapon Supply Interruption, missile feed failures.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>+2 dice</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>powerReroute</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>systemReset</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, and power-routing remedies. Helps reactor instability, power bus outage, shutdown recovery where appropriate.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Increase global machine shock/pressure capacity by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>+1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Ablative Module:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> drops to Resistance 1 at 50% armor remaining; destroyed at 25% armor remaining.</t>
+    </r>
+  </si>
+  <si>
+    <t>Armor &gt; 0</t>
+  </si>
+  <si>
+    <t>Gains High Emission (1) when Heat Status not SAFE</t>
+  </si>
+  <si>
+    <t>armorResistance</t>
+  </si>
+  <si>
+    <t>heatDissipation</t>
+  </si>
+  <si>
+    <t>heatBuffer</t>
+  </si>
+  <si>
+    <t>structure</t>
+  </si>
+  <si>
+    <t>remediation</t>
+  </si>
+  <si>
+    <t>Ready; not Prone/immobile; charge available</t>
+  </si>
+  <si>
+    <t>Ready; Structure remaining &lt; 100%</t>
+  </si>
+  <si>
+    <t>Immediately reduce heat, -5 heat</t>
+  </si>
+  <si>
+    <t>Consume on use</t>
+  </si>
+  <si>
+    <t>Heat &gt; 0; Coolant systems functional</t>
+  </si>
+  <si>
+    <t>At the start of the activation, recover 2 armor damage</t>
+  </si>
+  <si>
+    <t>10 charges then asset destroyed/consumed</t>
+  </si>
+  <si>
+    <t>Actuator Enhancement System</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">+3 DR; Grants </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Shield Block</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> reaction: Reduce incoming damage by 1</t>
+    </r>
+  </si>
+  <si>
+    <t>-5 AR for limb-mounted weapons; 5 Shield Block charges - asset disabled when out of charges</t>
+  </si>
+  <si>
+    <t>Ready; heat sinks functional</t>
+  </si>
+  <si>
+    <t>Ready</t>
+  </si>
+  <si>
+    <t>10 Charges</t>
+  </si>
+  <si>
+    <t>Incoming missile/cluster attack; charges available</t>
+  </si>
+  <si>
+    <t>Incoming missile/cluster attack</t>
+  </si>
+  <si>
+    <t>consumable</t>
+  </si>
+  <si>
+    <t>autoRepair, consumable</t>
+  </si>
+  <si>
+    <t>Free Action to jump 180 meters (or add +180 meters to a Jump Move)</t>
+  </si>
+  <si>
+    <t>1 charge, 3 turn recovery; Use generates +1 heat</t>
+  </si>
+  <si>
+    <t>High Emission (1) while in use, FA to sustain lock</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Target at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>contact</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or better; Line of Sight - successful TAG action</t>
+    </r>
+  </si>
+  <si>
+    <t>Target TAGged - Sensor Locked, generateTargetData against TAGged enemy is a Free Action</t>
+  </si>
+  <si>
+    <t>NARC Attack hits target; beacon attached</t>
+  </si>
+  <si>
+    <t>Attach NARC Beacon - NARCed target counts as Sensor Locked only for compatible guided missile systems., Beacon carrier trackingPenalty reduced by 3</t>
+  </si>
+  <si>
+    <t>UAV Active and not jammed</t>
+  </si>
+  <si>
+    <t>C3 Active</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Friendly C3 units may use the best friendly detection state on a target, capped at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>track</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> unless the attacker also has direct </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>lock</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. May use best shared targetingData packet from the network, not stacked.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>network</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>c3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>targetingData</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>sharedSensors</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>network</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>uav</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>remoteSensor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>eyeInSky</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>network</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>command</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>intelligence</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>initiative</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>coordination</t>
+    </r>
+  </si>
+  <si>
+    <t>Suppressed by IFF Jammer/network disruption</t>
+  </si>
+  <si>
+    <t>All friendly SLIC units have +1 initiative; Grants +1 die to acquireTarget, sensorSweep, holdLink, breakLock, generateTargetData to all friendly units within 500m</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Provides passive battlefield overwatch. Grants </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>+1 die</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Acquire Target / Sensor Sweep. Can maintain </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>contact</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> on visible enemies in UAV coverage. Grants +2 dice to Piloting checks to cross hazardous terrain/mine fields . Removes indirect fire penalties for operator.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3005,7 +3590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3056,17 +3641,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3075,6 +3658,27 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6752,58 +7356,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15.75" thickBot="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="31" t="s">
-        <v>270</v>
-      </c>
-      <c r="F1" s="31" t="s">
+      <c r="E1" s="29" t="s">
+        <v>268</v>
+      </c>
+      <c r="F1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="I1" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="31" t="s">
+      <c r="L1" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="M1" s="31" t="s">
+      <c r="M1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="31" t="s">
+      <c r="N1" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="O1" s="32" t="s">
+      <c r="O1" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="33" t="s">
+      <c r="P1" s="31" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16">
       <c r="B2" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="C2">
         <v>20</v>
@@ -6812,29 +7416,29 @@
         <v>128</v>
       </c>
       <c r="E2" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="B3" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="C3">
         <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="E3" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:16">
       <c r="B4" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="C4">
         <v>25</v>
@@ -6843,26 +7447,26 @@
         <v>130</v>
       </c>
       <c r="E4" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="B5" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="C5">
         <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="E5" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6" spans="1:16">
       <c r="B6" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="C6">
         <v>50</v>
@@ -6871,26 +7475,26 @@
         <v>132</v>
       </c>
       <c r="E6" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" spans="1:16">
       <c r="B7" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="C7">
         <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="E7" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="B8" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="C8">
         <v>65</v>
@@ -6899,12 +7503,12 @@
         <v>131</v>
       </c>
       <c r="E8" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="9" spans="1:16">
       <c r="B9" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="C9">
         <v>80</v>
@@ -6913,46 +7517,46 @@
         <v>131</v>
       </c>
       <c r="E9" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="B10" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="C10">
         <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="E10" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="B11" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="C11">
         <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="E11" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="B12" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="C12">
         <v>60</v>
@@ -6961,86 +7565,86 @@
         <v>130</v>
       </c>
       <c r="E12" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="A13" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="B13" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="C13">
         <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="E13" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="B14" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="C14">
         <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="E14" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="B15" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="C15">
         <v>1.5</v>
       </c>
       <c r="D15" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="E15" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="B16" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C16">
         <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="E16" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C17">
         <v>10</v>
       </c>
       <c r="D17" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="E17" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -7050,36 +7654,36 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4614B8F-CA9A-402E-B293-C8FF103E111E}">
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.42578125" customWidth="1"/>
-    <col min="4" max="4" width="50.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="108.42578125" style="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="61.28515625" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.42578125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="50.85546875" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="54.5703125" style="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="108.42578125" style="35" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="70.85546875" style="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="21" t="s">
-        <v>250</v>
+        <v>438</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
-        <v>305</v>
-      </c>
-      <c r="F1" s="26" t="s">
-        <v>304</v>
-      </c>
-      <c r="G1" s="26" t="s">
-        <v>311</v>
+      <c r="E1" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="F1" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="G1" s="33" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -7089,216 +7693,216 @@
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
       <c r="D2" s="28"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="3" spans="1:7">
       <c r="B3" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C3" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="D3" t="s">
-        <v>330</v>
-      </c>
-      <c r="E3" s="25" t="s">
+        <v>326</v>
+      </c>
+      <c r="E3" s="38" t="s">
+        <v>312</v>
+      </c>
+      <c r="F3" s="27" t="s">
         <v>316</v>
       </c>
-      <c r="F3" s="27" t="s">
-        <v>320</v>
-      </c>
-      <c r="G3" s="25" t="s">
-        <v>312</v>
+      <c r="G3" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="B4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C4" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="D4" t="s">
-        <v>331</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>317</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>309</v>
-      </c>
-      <c r="G4" s="25" t="s">
-        <v>312</v>
+        <v>327</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>313</v>
+      </c>
+      <c r="F4" s="35" t="s">
+        <v>305</v>
+      </c>
+      <c r="G4" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="B5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C5" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="D5" t="s">
-        <v>332</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>318</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>307</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>312</v>
+        <v>328</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="G5" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="B6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C6" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="D6" t="s">
-        <v>333</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>319</v>
-      </c>
-      <c r="F6" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>315</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>304</v>
+      </c>
+      <c r="G6" s="35" t="s">
         <v>308</v>
-      </c>
-      <c r="G6" s="25" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="28" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="28"/>
       <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
     </row>
     <row r="8" spans="1:7">
       <c r="B8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C8" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D8" t="s">
-        <v>334</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>312</v>
-      </c>
-      <c r="F8" s="25" t="s">
-        <v>314</v>
-      </c>
-      <c r="G8" s="25" t="s">
-        <v>313</v>
+        <v>330</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>308</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="B9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C9" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D9" t="s">
-        <v>334</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>312</v>
-      </c>
-      <c r="F9" s="25" t="s">
-        <v>315</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>313</v>
+        <v>330</v>
+      </c>
+      <c r="E9" s="38" t="s">
+        <v>308</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="G9" s="35" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="B10" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C10" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="D10" t="s">
-        <v>340</v>
-      </c>
-      <c r="E10" s="25" t="s">
-        <v>306</v>
-      </c>
-      <c r="F10" s="30" t="s">
-        <v>321</v>
-      </c>
-      <c r="G10" t="s">
-        <v>327</v>
+        <v>336</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>302</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>317</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="B11" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C11" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D11" t="s">
-        <v>335</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>310</v>
-      </c>
-      <c r="F11" s="25" t="s">
+        <v>331</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>306</v>
+      </c>
+      <c r="F11" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="G11" s="14" t="s">
         <v>322</v>
-      </c>
-      <c r="G11" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="B12" t="s">
-        <v>402</v>
+        <v>471</v>
       </c>
       <c r="C12" t="s">
-        <v>339</v>
-      </c>
-      <c r="E12" s="25" t="s">
-        <v>350</v>
-      </c>
-      <c r="F12" s="30" t="s">
-        <v>323</v>
-      </c>
-      <c r="G12" s="25" t="s">
-        <v>312</v>
+        <v>335</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>345</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>319</v>
+      </c>
+      <c r="G12" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="B13" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C13" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D13" t="s">
-        <v>342</v>
-      </c>
-      <c r="E13" s="25" t="s">
-        <v>310</v>
-      </c>
-      <c r="F13" s="30" t="s">
-        <v>324</v>
-      </c>
-      <c r="G13" t="s">
-        <v>325</v>
+        <v>338</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>306</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>320</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -7308,239 +7912,239 @@
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
       <c r="D14" s="28"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="E14" s="37"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+    </row>
+    <row r="15" spans="1:7" ht="30">
       <c r="B15" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C15" t="s">
-        <v>345</v>
-      </c>
-      <c r="D15" s="27" t="s">
-        <v>354</v>
-      </c>
-      <c r="E15" s="25" t="s">
-        <v>348</v>
-      </c>
-      <c r="F15" s="25" t="s">
-        <v>356</v>
-      </c>
-      <c r="G15" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>349</v>
+      </c>
+      <c r="E15" s="38" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="F15" s="35" t="s">
+        <v>351</v>
+      </c>
+      <c r="G15" s="35" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30">
       <c r="B16" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C16" t="s">
-        <v>345</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>355</v>
-      </c>
-      <c r="E16" s="25" t="s">
-        <v>348</v>
-      </c>
-      <c r="F16" s="25" t="s">
-        <v>357</v>
-      </c>
-      <c r="G16" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>350</v>
+      </c>
+      <c r="E16" s="38" t="s">
         <v>343</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>352</v>
+      </c>
+      <c r="G16" s="35" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="B17" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C17" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D17" t="s">
+        <v>342</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>346</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>348</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="30">
+      <c r="B18" t="s">
+        <v>291</v>
+      </c>
+      <c r="C18" t="s">
+        <v>340</v>
+      </c>
+      <c r="D18" s="26" t="s">
         <v>347</v>
       </c>
-      <c r="E17" t="s">
-        <v>351</v>
-      </c>
-      <c r="F17" s="25" t="s">
-        <v>353</v>
-      </c>
-      <c r="G17" s="25" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="B18" t="s">
-        <v>293</v>
-      </c>
-      <c r="C18" t="s">
-        <v>345</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>352</v>
-      </c>
-      <c r="E18" s="25" t="s">
-        <v>348</v>
-      </c>
-      <c r="F18" s="25" t="s">
-        <v>373</v>
-      </c>
-      <c r="G18" s="25" t="s">
-        <v>312</v>
+      <c r="E18" s="38" t="s">
+        <v>343</v>
+      </c>
+      <c r="F18" s="35" t="s">
+        <v>368</v>
+      </c>
+      <c r="G18" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="B19" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C19" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D19" t="s">
-        <v>349</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>348</v>
-      </c>
-      <c r="F19" s="25" t="s">
-        <v>358</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>359</v>
+        <v>344</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>343</v>
+      </c>
+      <c r="F19" s="35" t="s">
+        <v>353</v>
+      </c>
+      <c r="G19" s="35" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="28" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B20" s="28"/>
       <c r="C20" s="28"/>
       <c r="D20" s="28"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="E20" s="37"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+    </row>
+    <row r="21" spans="1:7" ht="45">
       <c r="B21" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C21" t="s">
-        <v>346</v>
-      </c>
-      <c r="D21" s="27" t="s">
+        <v>341</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>369</v>
+      </c>
+      <c r="F21" s="35" t="s">
+        <v>359</v>
+      </c>
+      <c r="G21" s="35" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="30">
+      <c r="B22" t="s">
+        <v>292</v>
+      </c>
+      <c r="C22" t="s">
+        <v>341</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>356</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>369</v>
+      </c>
+      <c r="F22" s="35" t="s">
         <v>360</v>
       </c>
-      <c r="E21" s="25" t="s">
-        <v>374</v>
-      </c>
-      <c r="F21" s="25" t="s">
+      <c r="G22" s="35" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="30">
+      <c r="B23" t="s">
+        <v>276</v>
+      </c>
+      <c r="C23" t="s">
+        <v>341</v>
+      </c>
+      <c r="D23" s="26" t="s">
+        <v>357</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>370</v>
+      </c>
+      <c r="F23" s="35" t="s">
+        <v>362</v>
+      </c>
+      <c r="G23" s="35" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="30">
+      <c r="B24" t="s">
+        <v>294</v>
+      </c>
+      <c r="C24" t="s">
+        <v>341</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>358</v>
+      </c>
+      <c r="E24" s="38" t="s">
+        <v>371</v>
+      </c>
+      <c r="F24" s="35" t="s">
+        <v>363</v>
+      </c>
+      <c r="G24" s="35" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="30">
+      <c r="B25" t="s">
+        <v>280</v>
+      </c>
+      <c r="C25" t="s">
+        <v>341</v>
+      </c>
+      <c r="D25" s="26" t="s">
+        <v>366</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>372</v>
+      </c>
+      <c r="F25" s="35" t="s">
         <v>364</v>
       </c>
-      <c r="G21" s="25" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="B22" t="s">
-        <v>294</v>
-      </c>
-      <c r="C22" t="s">
-        <v>346</v>
-      </c>
-      <c r="D22" s="27" t="s">
-        <v>361</v>
-      </c>
-      <c r="E22" s="25" t="s">
-        <v>374</v>
-      </c>
-      <c r="F22" s="25" t="s">
-        <v>365</v>
-      </c>
-      <c r="G22" s="25" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="B23" t="s">
-        <v>278</v>
-      </c>
-      <c r="C23" t="s">
-        <v>346</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>362</v>
-      </c>
-      <c r="E23" s="25" t="s">
-        <v>375</v>
-      </c>
-      <c r="F23" s="25" t="s">
-        <v>367</v>
-      </c>
-      <c r="G23" s="25" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="B24" t="s">
-        <v>296</v>
-      </c>
-      <c r="C24" t="s">
-        <v>346</v>
-      </c>
-      <c r="D24" s="27" t="s">
-        <v>363</v>
-      </c>
-      <c r="E24" s="25" t="s">
-        <v>376</v>
-      </c>
-      <c r="F24" s="25" t="s">
-        <v>368</v>
-      </c>
-      <c r="G24" s="25" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="B25" t="s">
-        <v>283</v>
-      </c>
-      <c r="C25" t="s">
-        <v>346</v>
-      </c>
-      <c r="D25" s="27" t="s">
-        <v>371</v>
-      </c>
-      <c r="E25" t="s">
-        <v>377</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>369</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>312</v>
+      <c r="G25" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="B26" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C26" t="s">
-        <v>346</v>
-      </c>
-      <c r="D26" s="27" t="s">
-        <v>370</v>
-      </c>
-      <c r="E26" s="25" t="s">
-        <v>378</v>
-      </c>
-      <c r="F26" s="25" t="s">
-        <v>372</v>
-      </c>
-      <c r="G26" s="25" t="s">
-        <v>344</v>
+        <v>341</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>365</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>373</v>
+      </c>
+      <c r="F26" s="35" t="s">
+        <v>367</v>
+      </c>
+      <c r="G26" s="35" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -7550,317 +8154,527 @@
       <c r="B27" s="28"/>
       <c r="C27" s="28"/>
       <c r="D27" s="28"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="E27" s="37"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
+    </row>
+    <row r="28" spans="1:7" ht="30">
       <c r="B28" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C28" t="s">
-        <v>399</v>
-      </c>
-      <c r="D28" s="27" t="s">
-        <v>382</v>
-      </c>
-      <c r="E28" t="s">
-        <v>380</v>
-      </c>
-      <c r="F28" s="25" t="s">
-        <v>386</v>
-      </c>
-      <c r="G28" t="s">
+        <v>394</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>377</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>375</v>
+      </c>
+      <c r="F28" s="35" t="s">
         <v>381</v>
+      </c>
+      <c r="G28" s="14" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="B29" t="s">
+        <v>374</v>
+      </c>
+      <c r="C29" t="s">
+        <v>394</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>378</v>
+      </c>
+      <c r="E29" s="24" t="s">
         <v>379</v>
       </c>
-      <c r="C29" t="s">
-        <v>399</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>383</v>
-      </c>
-      <c r="E29" t="s">
-        <v>384</v>
-      </c>
-      <c r="F29" s="25" t="s">
-        <v>385</v>
-      </c>
-      <c r="G29" s="25" t="s">
-        <v>312</v>
+      <c r="F29" s="35" t="s">
+        <v>380</v>
+      </c>
+      <c r="G29" s="35" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="28" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B30" s="28"/>
       <c r="C30" s="28"/>
       <c r="D30" s="28"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="29"/>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="E30" s="37"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
+    </row>
+    <row r="31" spans="1:7" ht="30">
       <c r="B31" t="s">
+        <v>387</v>
+      </c>
+      <c r="C31" t="s">
+        <v>395</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>382</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>385</v>
+      </c>
+      <c r="F31" s="35" t="s">
         <v>392</v>
       </c>
-      <c r="C31" t="s">
-        <v>400</v>
-      </c>
-      <c r="D31" s="27" t="s">
-        <v>387</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="G31" s="14" t="s">
         <v>390</v>
-      </c>
-      <c r="F31" s="25" t="s">
-        <v>397</v>
-      </c>
-      <c r="G31" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="B32" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C32" t="s">
-        <v>400</v>
-      </c>
-      <c r="D32" s="27" t="s">
+        <v>395</v>
+      </c>
+      <c r="D32" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>385</v>
+      </c>
+      <c r="F32" s="35" t="s">
+        <v>388</v>
+      </c>
+      <c r="G32" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="E32" t="s">
-        <v>390</v>
-      </c>
-      <c r="F32" s="25" t="s">
+    </row>
+    <row r="33" spans="1:7" ht="45">
+      <c r="B33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C33" t="s">
+        <v>396</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>383</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>386</v>
+      </c>
+      <c r="F33" s="36" t="s">
         <v>393</v>
       </c>
-      <c r="G32" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="B33" t="s">
-        <v>289</v>
-      </c>
-      <c r="C33" t="s">
-        <v>401</v>
-      </c>
-      <c r="D33" s="27" t="s">
-        <v>388</v>
-      </c>
-      <c r="E33" t="s">
+      <c r="G33" s="14" t="s">
         <v>391</v>
-      </c>
-      <c r="F33" s="30" t="s">
-        <v>398</v>
-      </c>
-      <c r="G33" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="28" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B34" s="28"/>
       <c r="C34" s="28"/>
       <c r="D34" s="28"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="29"/>
-      <c r="G34" s="29"/>
-    </row>
-    <row r="35" spans="1:7">
+      <c r="E34" s="37"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+    </row>
+    <row r="35" spans="1:7" ht="30">
       <c r="B35" t="s">
-        <v>261</v>
-      </c>
-      <c r="E35" s="25"/>
-    </row>
-    <row r="36" spans="1:7">
+        <v>259</v>
+      </c>
+      <c r="D35" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="E35" s="38" t="s">
+        <v>489</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="45">
       <c r="B36" t="s">
-        <v>297</v>
-      </c>
-      <c r="E36" s="25"/>
-    </row>
-    <row r="37" spans="1:7">
+        <v>443</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>492</v>
+      </c>
+      <c r="E36" s="38" t="s">
+        <v>488</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="30">
       <c r="B37" t="s">
-        <v>292</v>
-      </c>
-      <c r="E37" s="25"/>
+        <v>290</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>493</v>
+      </c>
+      <c r="E37" s="38"/>
+      <c r="F37" s="35" t="s">
+        <v>495</v>
+      </c>
+      <c r="G37" s="24" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="28" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B38" s="28"/>
       <c r="C38" s="28"/>
       <c r="D38" s="28"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-    </row>
-    <row r="39" spans="1:7">
+      <c r="E38" s="37"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
+    </row>
+    <row r="39" spans="1:7" ht="30">
       <c r="B39" t="s">
-        <v>266</v>
-      </c>
-      <c r="E39" s="25"/>
-    </row>
-    <row r="40" spans="1:7">
+        <v>264</v>
+      </c>
+      <c r="D39" t="s">
+        <v>479</v>
+      </c>
+      <c r="E39" s="24" t="s">
+        <v>450</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="G39" s="14" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="30">
       <c r="B40" t="s">
+        <v>265</v>
+      </c>
+      <c r="D40" t="s">
+        <v>463</v>
+      </c>
+      <c r="E40" s="38"/>
+      <c r="F40" s="27" t="s">
+        <v>453</v>
+      </c>
+      <c r="G40" s="35" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="30">
+      <c r="B41" t="s">
         <v>267</v>
       </c>
-      <c r="E40" s="25"/>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="B41" t="s">
-        <v>269</v>
-      </c>
-      <c r="E41" s="25"/>
+      <c r="D41" t="s">
+        <v>463</v>
+      </c>
+      <c r="E41" s="38"/>
+      <c r="F41" s="27" t="s">
+        <v>454</v>
+      </c>
+      <c r="G41" s="35" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="42" spans="1:7">
       <c r="B42" t="s">
-        <v>281</v>
-      </c>
-      <c r="E42" s="25"/>
+        <v>442</v>
+      </c>
+      <c r="D42" t="s">
+        <v>462</v>
+      </c>
+      <c r="E42" s="38"/>
+      <c r="F42" s="14" t="s">
+        <v>455</v>
+      </c>
+      <c r="G42" s="35" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="43" spans="1:7">
       <c r="B43" t="s">
-        <v>285</v>
-      </c>
-      <c r="E43" s="25"/>
+        <v>283</v>
+      </c>
+      <c r="D43" t="s">
+        <v>461</v>
+      </c>
+      <c r="E43" s="38"/>
+      <c r="F43" s="35" t="s">
+        <v>433</v>
+      </c>
+      <c r="G43" s="35" t="s">
+        <v>458</v>
+      </c>
     </row>
     <row r="44" spans="1:7">
       <c r="B44" t="s">
-        <v>300</v>
-      </c>
-      <c r="E44" s="25"/>
-    </row>
-    <row r="45" spans="1:7">
+        <v>282</v>
+      </c>
+      <c r="D44" t="s">
+        <v>460</v>
+      </c>
+      <c r="E44" s="38"/>
+      <c r="F44" s="35" t="s">
+        <v>434</v>
+      </c>
+      <c r="G44" s="35" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="30">
       <c r="B45" t="s">
-        <v>303</v>
-      </c>
-      <c r="E45" s="25"/>
-    </row>
-    <row r="46" spans="1:7">
+        <v>296</v>
+      </c>
+      <c r="D45" t="s">
+        <v>459</v>
+      </c>
+      <c r="E45" s="24" t="s">
+        <v>457</v>
+      </c>
+      <c r="F45" s="35" t="s">
+        <v>435</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="30">
       <c r="B46" t="s">
-        <v>298</v>
-      </c>
-      <c r="E46" s="25"/>
-    </row>
-    <row r="47" spans="1:7">
+        <v>299</v>
+      </c>
+      <c r="D46" t="s">
+        <v>459</v>
+      </c>
+      <c r="E46" s="24" t="s">
+        <v>457</v>
+      </c>
+      <c r="F46" s="35" t="s">
+        <v>436</v>
+      </c>
+      <c r="G46" s="15" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="30">
       <c r="B47" t="s">
-        <v>299</v>
-      </c>
-      <c r="E47" s="25"/>
+        <v>295</v>
+      </c>
+      <c r="D47" t="s">
+        <v>459</v>
+      </c>
+      <c r="E47" s="24" t="s">
+        <v>457</v>
+      </c>
+      <c r="F47" s="35" t="s">
+        <v>437</v>
+      </c>
+      <c r="G47" s="15" t="s">
+        <v>456</v>
+      </c>
     </row>
     <row r="48" spans="1:7">
-      <c r="E48" s="25"/>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" s="21" t="s">
+      <c r="B48" t="s">
+        <v>297</v>
+      </c>
+      <c r="D48" t="s">
+        <v>480</v>
+      </c>
+      <c r="E48" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="F48" s="35" t="s">
+        <v>469</v>
+      </c>
+      <c r="G48" s="35" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="32" t="s">
+        <v>255</v>
+      </c>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="34"/>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="B50" t="s">
+        <v>274</v>
+      </c>
+      <c r="D50" s="25"/>
+      <c r="E50" s="24" t="s">
+        <v>484</v>
+      </c>
+      <c r="F50" s="35" t="s">
+        <v>485</v>
+      </c>
+      <c r="G50" s="35" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="30">
+      <c r="B51" t="s">
+        <v>275</v>
+      </c>
+      <c r="D51" s="25" t="s">
+        <v>479</v>
+      </c>
+      <c r="E51" s="24" t="s">
+        <v>486</v>
+      </c>
+      <c r="F51" s="35" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="B52" t="s">
+        <v>281</v>
+      </c>
+      <c r="D52" s="25" t="s">
+        <v>479</v>
+      </c>
+      <c r="E52" s="24" t="s">
+        <v>464</v>
+      </c>
+      <c r="F52" s="35" t="s">
+        <v>481</v>
+      </c>
+      <c r="G52" s="35" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="B53" t="s">
+        <v>266</v>
+      </c>
+      <c r="D53" s="25" t="s">
+        <v>479</v>
+      </c>
+      <c r="E53" s="24" t="s">
+        <v>468</v>
+      </c>
+      <c r="F53" s="35" t="s">
+        <v>466</v>
+      </c>
+      <c r="G53" s="35" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="30">
+      <c r="B54" t="s">
+        <v>289</v>
+      </c>
+      <c r="D54" s="25"/>
+      <c r="E54" s="24" t="s">
+        <v>475</v>
+      </c>
+      <c r="F54" s="35" t="s">
+        <v>472</v>
+      </c>
+      <c r="G54" s="35" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="B55" t="s">
+        <v>441</v>
+      </c>
+      <c r="E55" s="24" t="s">
+        <v>474</v>
+      </c>
+      <c r="F55" s="35" t="s">
+        <v>432</v>
+      </c>
+      <c r="G55" s="35" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="B56" t="s">
+        <v>439</v>
+      </c>
+      <c r="D56" s="25"/>
+      <c r="E56" s="24" t="s">
+        <v>477</v>
+      </c>
+      <c r="F56" s="35" t="s">
+        <v>444</v>
+      </c>
+      <c r="G56" s="35" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="B57" t="s">
+        <v>440</v>
+      </c>
+      <c r="E57" s="24" t="s">
+        <v>478</v>
+      </c>
+      <c r="F57" s="35" t="s">
+        <v>444</v>
+      </c>
+      <c r="G57" s="35" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="D58" s="25"/>
+      <c r="E58" s="38"/>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="D59" s="25"/>
+      <c r="E59" s="38"/>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="E60" s="38"/>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" s="21" t="s">
+        <v>431</v>
+      </c>
+      <c r="E61" s="38"/>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="B62" t="s">
+        <v>250</v>
+      </c>
+      <c r="F62" s="14"/>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="B63" t="s">
         <v>251</v>
       </c>
-      <c r="E49" s="25"/>
-    </row>
-    <row r="50" spans="1:5">
-      <c r="A50" t="s">
+      <c r="E63" s="38"/>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="B64" t="s">
         <v>252</v>
       </c>
-      <c r="E50" s="25"/>
-    </row>
-    <row r="51" spans="1:5">
-      <c r="A51" t="s">
+      <c r="E64" s="38"/>
+    </row>
+    <row r="65" spans="2:5">
+      <c r="B65" t="s">
         <v>253</v>
       </c>
-      <c r="E51" s="25"/>
-    </row>
-    <row r="52" spans="1:5">
-      <c r="A52" t="s">
+      <c r="E65" s="38"/>
+    </row>
+    <row r="66" spans="2:5">
+      <c r="B66" t="s">
         <v>254</v>
       </c>
-      <c r="E52" s="25"/>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="A53" t="s">
-        <v>255</v>
-      </c>
-      <c r="E53" s="25"/>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" t="s">
-        <v>256</v>
-      </c>
-      <c r="E54" s="25"/>
-    </row>
-    <row r="55" spans="1:5">
-      <c r="E55" s="25"/>
-    </row>
-    <row r="56" spans="1:5">
-      <c r="E56" s="25"/>
-    </row>
-    <row r="57" spans="1:5">
-      <c r="E57" s="25"/>
-    </row>
-    <row r="58" spans="1:5">
-      <c r="E58" s="25"/>
-    </row>
-    <row r="59" spans="1:5">
-      <c r="E59" s="25"/>
-    </row>
-    <row r="60" spans="1:5">
-      <c r="E60" s="25"/>
-    </row>
-    <row r="61" spans="1:5">
-      <c r="E61" s="25"/>
-    </row>
-    <row r="62" spans="1:5">
-      <c r="E62" s="25"/>
-    </row>
-    <row r="63" spans="1:5">
-      <c r="A63" s="24" t="s">
-        <v>257</v>
-      </c>
-      <c r="E63" s="25"/>
-    </row>
-    <row r="64" spans="1:5">
-      <c r="A64" t="s">
-        <v>276</v>
-      </c>
-      <c r="E64" s="25"/>
-    </row>
-    <row r="65" spans="1:5">
-      <c r="A65" t="s">
-        <v>277</v>
-      </c>
-      <c r="E65" s="25"/>
-    </row>
-    <row r="66" spans="1:5">
-      <c r="A66" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5">
-      <c r="A67" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5">
-      <c r="A68" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5">
-      <c r="A69" t="s">
-        <v>301</v>
-      </c>
+      <c r="E66" s="38"/>
     </row>
   </sheetData>
+  <dataConsolidate/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8301,8 +9115,11 @@
       <c r="C16" s="22" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="17" spans="1:11">
+      <c r="K16" s="14" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" t="s">
         <v>236</v>
       </c>
@@ -8312,8 +9129,14 @@
       <c r="C17" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="18" spans="1:11">
+      <c r="K17" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="L17" s="25" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18" t="s">
         <v>237</v>
       </c>
@@ -8324,7 +9147,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:12">
       <c r="B19" t="s">
         <v>241</v>
       </c>
@@ -8332,7 +9155,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:12">
       <c r="A20" t="s">
         <v>240</v>
       </c>
@@ -8351,7 +9174,7 @@
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:12">
       <c r="B21" t="s">
         <v>241</v>
       </c>
@@ -8367,7 +9190,7 @@
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:12">
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
       <c r="F22" s="14"/>
@@ -8377,7 +9200,7 @@
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:12">
       <c r="D23" s="15"/>
       <c r="E23" s="15"/>
       <c r="F23" s="14"/>
@@ -8387,7 +9210,7 @@
       <c r="J23" s="14"/>
       <c r="K23" s="14"/>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:12">
       <c r="D24" s="15"/>
       <c r="E24" s="15"/>
       <c r="F24" s="14"/>
@@ -8397,7 +9220,7 @@
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:12">
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
       <c r="F25" s="14"/>
@@ -8407,7 +9230,7 @@
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:12">
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
       <c r="F26" s="14"/>
@@ -8417,7 +9240,7 @@
       <c r="J26" s="14"/>
       <c r="K26" s="14"/>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:12">
       <c r="D27" s="15"/>
       <c r="E27" s="15"/>
       <c r="F27" s="14"/>
@@ -8427,7 +9250,7 @@
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:12">
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
       <c r="F28" s="14"/>
@@ -8437,7 +9260,7 @@
       <c r="J28" s="14"/>
       <c r="K28" s="14"/>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:12">
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
       <c r="F29" s="14"/>
@@ -8447,7 +9270,7 @@
       <c r="J29" s="14"/>
       <c r="K29" s="14"/>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:12">
       <c r="D30" s="15"/>
       <c r="E30" s="15"/>
       <c r="F30" s="14"/>
@@ -8457,7 +9280,7 @@
       <c r="J30" s="14"/>
       <c r="K30" s="14"/>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:12">
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
       <c r="F31" s="14"/>
@@ -8467,7 +9290,7 @@
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:12">
       <c r="D32" s="15"/>
       <c r="E32" s="15"/>
       <c r="F32" s="14"/>

</xml_diff>